<commit_message>
Separa Repuestos/Modelo de Unidades, actualiza inputs y agrega reglas de NPF
- Página intermedia para elegir Repuestos o Modelo de Unidades (/ampliar/<tipo>),
  botones "volver" y rediseño con radios/sombras más suaves.
- Modelo de Unidades habilitado y renombrado; input por nombre (como Repuestos)
  desde plantilla_modelos.xlsx; TIPO MATERIAL define plantilla y rango
  (ZVEH 10M, ZMAQ 20M, ZCAM 30M, ZUSA 40M). ZVHE renombrado a ZVEH; nueva
  plantilla SAP ZUSA.
- Repuestos: columna opcional "Codigo antiguo" (col. AL, con NPF de respaldo).
- Regla NPF: si supera 18 caracteres se usa el correlativo; si NPF:Fabricante
  (con el Fabricante externo, ej. DFAC) ya existe en BaseDatosRepuestos.xlsx o
  se repite en el archivo, el correlativo va en el EAN.
- Se quita del formulario el texto sobre la hoja PENDIENTES (nunca se generaba).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/reference/Repuestos/plantilla_repuestos.xlsx
+++ b/data/reference/Repuestos/plantilla_repuestos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tattersall-my.sharepoint.com/personal/sherrera_tattersall_cl/Documents/Escritorio/FACU/INPUTS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="204" documentId="13_ncr:1_{E4143A50-A376-493D-8BAE-F5574D41C3D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{158801E5-C6C0-4551-B525-D2EDD3D15A77}"/>
+  <xr:revisionPtr revIDLastSave="213" documentId="13_ncr:1_{E4143A50-A376-493D-8BAE-F5574D41C3D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE1E1106-E0DF-419F-95E5-8914EDD20E84}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="775" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="775" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Input" sheetId="1" r:id="rId1"/>
@@ -68,7 +68,7 @@
     A esto, debemos hacerle .upper() para asegurar que quede todo en mayuscula (en el código)</t>
       </text>
     </comment>
-    <comment ref="H1" authorId="2" shapeId="0" xr:uid="{AB502CC6-540A-4EFE-BE2E-13D893D1B339}">
+    <comment ref="I1" authorId="2" shapeId="0" xr:uid="{AB502CC6-540A-4EFE-BE2E-13D893D1B339}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -78,7 +78,7 @@
 elif len(NPF) &lt;= 18: EAN = NPF</t>
       </text>
     </comment>
-    <comment ref="L1" authorId="3" shapeId="0" xr:uid="{FCED281E-191C-464F-A9DE-B59B7386F380}">
+    <comment ref="M1" authorId="3" shapeId="0" xr:uid="{FCED281E-191C-464F-A9DE-B59B7386F380}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -93,7 +93,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12494" uniqueCount="2985">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12495" uniqueCount="2986">
   <si>
     <t>NPF</t>
   </si>
@@ -9048,6 +9048,9 @@
   </si>
   <si>
     <t>10.99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Codigo antiguo </t>
   </si>
 </sst>
 </file>
@@ -9186,7 +9189,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -9227,9 +9230,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9556,12 +9556,12 @@
   <threadedComment ref="E1" dT="2026-09-14T16:05:23.90" personId="{171AD741-F941-45FC-832C-2B82E3AD0F23}" id="{7ED35A56-13BB-4556-B92E-66A09D00C913}">
     <text>A esto, debemos hacerle .upper() para asegurar que quede todo en mayuscula (en el código)</text>
   </threadedComment>
-  <threadedComment ref="H1" dT="2026-09-14T16:04:55.44" personId="{171AD741-F941-45FC-832C-2B82E3AD0F23}" id="{AB502CC6-540A-4EFE-BE2E-13D893D1B339}">
+  <threadedComment ref="I1" dT="2026-09-14T16:04:55.44" personId="{171AD741-F941-45FC-832C-2B82E3AD0F23}" id="{AB502CC6-540A-4EFE-BE2E-13D893D1B339}">
     <text>Con el NPF se calcula el EAN:
 If len(NPF) &gt; 18: EAN = Correlativo
 elif len(NPF) &lt;= 18: EAN = NPF</text>
   </threadedComment>
-  <threadedComment ref="L1" dT="2026-09-14T16:00:42.01" personId="{171AD741-F941-45FC-832C-2B82E3AD0F23}" id="{FCED281E-191C-464F-A9DE-B59B7386F380}">
+  <threadedComment ref="M1" dT="2026-09-14T16:00:42.01" personId="{171AD741-F941-45FC-832C-2B82E3AD0F23}" id="{FCED281E-191C-464F-A9DE-B59B7386F380}">
     <text>Validaciones:
 Si Moneda == CLP -&gt; Int(Costo unitario)
 Else -&gt; float (Costo unitario)</text>
@@ -9571,7 +9571,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -9580,17 +9580,18 @@
     <col min="4" max="4" width="14" style="1" customWidth="1"/>
     <col min="5" max="5" width="44.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18" style="1" customWidth="1"/>
-    <col min="8" max="8" width="14" style="24" customWidth="1"/>
-    <col min="9" max="9" width="22" style="1" customWidth="1"/>
-    <col min="10" max="10" width="14" style="1" customWidth="1"/>
-    <col min="11" max="11" width="19" style="1" customWidth="1"/>
-    <col min="12" max="12" width="25.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="9.140625" style="1"/>
+    <col min="7" max="7" width="68.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18" style="1" customWidth="1"/>
+    <col min="9" max="9" width="14" style="24" customWidth="1"/>
+    <col min="10" max="10" width="22" style="1" customWidth="1"/>
+    <col min="11" max="11" width="14" style="1" customWidth="1"/>
+    <col min="12" max="12" width="19" style="1" customWidth="1"/>
+    <col min="13" max="13" width="25.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>2954</v>
       </c>
@@ -9612,26 +9613,29 @@
       <c r="G1" s="5" t="s">
         <v>2887</v>
       </c>
-      <c r="H1" s="22" t="s">
+      <c r="H1" s="5" t="s">
+        <v>2985</v>
+      </c>
+      <c r="I1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>2959</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>2960</v>
       </c>
     </row>
-    <row r="2" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>2891</v>
       </c>
@@ -9641,35 +9645,36 @@
       <c r="D2" s="2" t="s">
         <v>2885</v>
       </c>
-      <c r="E2" s="26" t="s">
+      <c r="E2" s="3" t="s">
         <v>2866</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>357</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>1697</v>
-      </c>
-      <c r="H2" s="23" t="s">
+        <v>1045</v>
+      </c>
+      <c r="H2" s="3"/>
+      <c r="I2" s="23" t="s">
         <v>2868</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>18</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>73</v>
       </c>
       <c r="K2" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="M2" s="2" t="s">
         <v>2957</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>2958</v>
       </c>
     </row>
-    <row r="3" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>2891</v>
       </c>
@@ -9679,7 +9684,7 @@
       <c r="D3" s="2" t="s">
         <v>2885</v>
       </c>
-      <c r="E3" s="26" t="s">
+      <c r="E3" s="3" t="s">
         <v>2869</v>
       </c>
       <c r="F3" s="3" t="s">
@@ -9688,26 +9693,27 @@
       <c r="G3" s="4" t="s">
         <v>1079</v>
       </c>
-      <c r="H3" s="23" t="s">
+      <c r="H3" s="3"/>
+      <c r="I3" s="23" t="s">
         <v>2871</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="J3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="K3" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="L3" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="M3" s="2" t="s">
         <v>2984</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="N3" s="2" t="s">
         <v>2958</v>
       </c>
     </row>
-    <row r="4" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2891</v>
       </c>
@@ -9717,7 +9723,7 @@
       <c r="D4" s="2" t="s">
         <v>2885</v>
       </c>
-      <c r="E4" s="26" t="s">
+      <c r="E4" s="3" t="s">
         <v>2872</v>
       </c>
       <c r="F4" s="3" t="s">
@@ -9726,26 +9732,27 @@
       <c r="G4" s="4" t="s">
         <v>1364</v>
       </c>
-      <c r="H4" s="23" t="s">
+      <c r="H4" s="3"/>
+      <c r="I4" s="23" t="s">
         <v>2874</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="J4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="K4" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="K4" s="4" t="s">
+      <c r="L4" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="M4" s="2" t="s">
         <v>2982</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="N4" s="2" t="s">
         <v>2981</v>
       </c>
     </row>
-    <row r="5" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>2891</v>
       </c>
@@ -9755,7 +9762,7 @@
       <c r="D5" s="2" t="s">
         <v>2885</v>
       </c>
-      <c r="E5" s="26" t="s">
+      <c r="E5" s="3" t="s">
         <v>2875</v>
       </c>
       <c r="F5" s="3" t="s">
@@ -9764,26 +9771,27 @@
       <c r="G5" s="4" t="s">
         <v>1534</v>
       </c>
-      <c r="H5" s="23" t="s">
+      <c r="H5" s="3"/>
+      <c r="I5" s="23" t="s">
         <v>2876</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="J5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="K5" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="L5" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="M5" s="2" t="s">
         <v>2978</v>
       </c>
-      <c r="M5" s="2" t="s">
+      <c r="N5" s="2" t="s">
         <v>2958</v>
       </c>
     </row>
-    <row r="6" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>2891</v>
       </c>
@@ -9793,7 +9801,7 @@
       <c r="D6" s="2" t="s">
         <v>2885</v>
       </c>
-      <c r="E6" s="26" t="s">
+      <c r="E6" s="3" t="s">
         <v>2877</v>
       </c>
       <c r="F6" s="3" t="s">
@@ -9802,26 +9810,27 @@
       <c r="G6" s="4" t="s">
         <v>1674</v>
       </c>
-      <c r="H6" s="23" t="s">
+      <c r="H6" s="3"/>
+      <c r="I6" s="23" t="s">
         <v>2878</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="J6" s="4" t="s">
         <v>18</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>73</v>
       </c>
       <c r="K6" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="L6" s="2" t="s">
+      <c r="L6" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="M6" s="2" t="s">
         <v>2979</v>
       </c>
-      <c r="M6" s="2" t="s">
+      <c r="N6" s="2" t="s">
         <v>2958</v>
       </c>
     </row>
-    <row r="7" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>2891</v>
       </c>
@@ -9831,7 +9840,7 @@
       <c r="D7" s="2" t="s">
         <v>2885</v>
       </c>
-      <c r="E7" s="26" t="s">
+      <c r="E7" s="3" t="s">
         <v>2879</v>
       </c>
       <c r="F7" s="3" t="s">
@@ -9840,26 +9849,27 @@
       <c r="G7" s="4" t="s">
         <v>1147</v>
       </c>
-      <c r="H7" s="23" t="s">
+      <c r="H7" s="3"/>
+      <c r="I7" s="23" t="s">
         <v>2881</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="J7" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="K7" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="K7" s="4" t="s">
+      <c r="L7" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="M7" s="2" t="s">
         <v>2980</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="N7" s="2" t="s">
         <v>2958</v>
       </c>
     </row>
-    <row r="8" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>2891</v>
       </c>
@@ -9869,7 +9879,7 @@
       <c r="D8" s="2" t="s">
         <v>2885</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="E8" s="3" t="s">
         <v>2882</v>
       </c>
       <c r="F8" s="3" t="s">
@@ -9878,22 +9888,23 @@
       <c r="G8" s="4" t="s">
         <v>1883</v>
       </c>
-      <c r="H8" s="23" t="s">
+      <c r="H8" s="3"/>
+      <c r="I8" s="23" t="s">
         <v>2883</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="J8" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="K8" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="L8" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="M8" s="2" t="s">
         <v>2983</v>
       </c>
-      <c r="M8" s="2" t="s">
+      <c r="N8" s="2" t="s">
         <v>2981</v>
       </c>
     </row>
@@ -9906,10 +9917,10 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B1048576" xr:uid="{3831DDEE-9479-489B-9FF5-DEBDD2CDE240}">
       <formula1>"UN,L"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2:M1048576" xr:uid="{6F6504BA-302F-4A71-8913-44DB499E65AF}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:N1048576" xr:uid="{6F6504BA-302F-4A71-8913-44DB499E65AF}">
       <formula1>"CLP,USD"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:K1048576" xr:uid="{A4E5013D-F794-4B1C-9E6D-EE2050F8FE69}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:L1048576" xr:uid="{A4E5013D-F794-4B1C-9E6D-EE2050F8FE69}">
       <formula1>#REF!</formula1>
     </dataValidation>
   </dataValidations>
@@ -9929,7 +9940,7 @@
           <x14:formula1>
             <xm:f>'Diccionario Original-Alternativ'!$B$2:$B$3</xm:f>
           </x14:formula1>
-          <xm:sqref>I2:I1048576</xm:sqref>
+          <xm:sqref>J2:J1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{6888CB7A-8B50-4816-8706-E5D50FD7E731}">
           <x14:formula1>

</xml_diff>